<commit_message>
Fix: Case-insensitive matching for Amharic metadata fields and add debug logging
</commit_message>
<xml_diff>
--- a/Tender_3_Groups.xlsx
+++ b/Tender_3_Groups.xlsx
@@ -11,7 +11,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="116">
+  <si>
+    <t>Tender Number</t>
+  </si>
+  <si>
+    <t>033/2018</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>የተለያዩ የምግብነኮች</t>
+  </si>
   <si>
     <t>የተያዘበት ቀን</t>
   </si>
@@ -25,19 +37,13 @@
     <t>ከሀረር</t>
   </si>
   <si>
-    <t>Tender Number</t>
-  </si>
-  <si>
-    <t>033/2018</t>
+    <t>ያዥው አካል</t>
+  </si>
+  <si>
+    <t>Dire Dawa Customs Commission</t>
   </si>
   <si>
     <t>Exchange Rate</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>የተለያዩ የምግብነኮች</t>
   </si>
   <si>
     <t>ኮድ</t>
@@ -788,80 +794,88 @@
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
-        <v>157.098</v>
+      <c r="B4" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>157.098</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F8" s="3">
         <v>25</v>
@@ -882,7 +896,7 @@
         <v>103802.5</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M8" s="3">
         <v>25</v>
@@ -896,19 +910,19 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F9" s="3">
         <v>11</v>
@@ -929,7 +943,7 @@
         <v>6843.19</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M9" s="3">
         <v>25</v>
@@ -943,19 +957,19 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F10" s="3">
         <v>6</v>
@@ -976,7 +990,7 @@
         <v>15571.55</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M10" s="3">
         <v>25</v>
@@ -990,19 +1004,19 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F11" s="3">
         <v>18</v>
@@ -1023,7 +1037,7 @@
         <v>43688.95</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M11" s="3">
         <v>25</v>
@@ -1037,19 +1051,19 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="F12" s="3">
         <v>11</v>
@@ -1070,7 +1084,7 @@
         <v>26698.81</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M12" s="3">
         <v>25</v>
@@ -1084,19 +1098,19 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F13" s="3">
         <v>1</v>
@@ -1117,7 +1131,7 @@
         <v>2427.16</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M13" s="3">
         <v>25</v>
@@ -1131,19 +1145,19 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="F14" s="3">
         <v>4</v>
@@ -1164,7 +1178,7 @@
         <v>19423.6</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M14" s="3">
         <v>25</v>
@@ -1178,19 +1192,19 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F15" s="3">
         <v>7</v>
@@ -1211,7 +1225,7 @@
         <v>14878.75</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="M15" s="3">
         <v>25</v>
@@ -1225,19 +1239,19 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F16" s="3">
         <v>16</v>
@@ -1258,7 +1272,7 @@
         <v>58088.56</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M16" s="3">
         <v>25</v>
@@ -1272,19 +1286,19 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="F17" s="3">
         <v>1</v>
@@ -1305,7 +1319,7 @@
         <v>1955.87</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M17" s="3">
         <v>25</v>
@@ -1319,19 +1333,19 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F18" s="3">
         <v>47</v>
@@ -1352,7 +1366,7 @@
         <v>18311.34</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M18" s="3">
         <v>25</v>
@@ -1366,19 +1380,19 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F19" s="3">
         <v>3</v>
@@ -1399,7 +1413,7 @@
         <v>2262.21</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M19" s="3">
         <v>25</v>
@@ -1413,19 +1427,19 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F20" s="3">
         <v>6</v>
@@ -1446,7 +1460,7 @@
         <v>5278.49</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M20" s="3">
         <v>25</v>
@@ -1460,19 +1474,19 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F21" s="3">
         <v>6</v>
@@ -1493,7 +1507,7 @@
         <v>4383.03</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M21" s="3">
         <v>25</v>
@@ -1507,19 +1521,19 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F22" s="3">
         <v>12</v>
@@ -1540,7 +1554,7 @@
         <v>20680.38</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M22" s="3">
         <v>25</v>
@@ -1554,19 +1568,19 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F23" s="3">
         <v>5</v>
@@ -1587,7 +1601,7 @@
         <v>10949.73</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M23" s="3">
         <v>25</v>
@@ -1601,19 +1615,19 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F24" s="3">
         <v>6</v>
@@ -1634,7 +1648,7 @@
         <v>10340.19</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M24" s="3">
         <v>25</v>
@@ -1648,19 +1662,19 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F25" s="3">
         <v>5</v>
@@ -1681,7 +1695,7 @@
         <v>2984.86</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M25" s="3">
         <v>25</v>
@@ -1695,19 +1709,19 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F26" s="3">
         <v>22</v>
@@ -1728,7 +1742,7 @@
         <v>3628.96</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M26" s="3">
         <v>25</v>
@@ -1742,19 +1756,19 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="F27" s="3">
         <v>277</v>
@@ -1775,7 +1789,7 @@
         <v>53524.86</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M27" s="3">
         <v>25</v>
@@ -1789,19 +1803,19 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F28" s="3">
         <v>18</v>
@@ -1822,7 +1836,7 @@
         <v>3478.15</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M28" s="3">
         <v>25</v>
@@ -1836,19 +1850,19 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F29" s="3">
         <v>38</v>
@@ -1869,7 +1883,7 @@
         <v>8059.13</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M29" s="3">
         <v>25</v>
@@ -1883,19 +1897,19 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F30" s="3">
         <v>37</v>
@@ -1916,7 +1930,7 @@
         <v>7149.53</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M30" s="3">
         <v>22</v>
@@ -1930,19 +1944,19 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F31" s="3">
         <v>397</v>
@@ -1963,7 +1977,7 @@
         <v>76712.52</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M31" s="3">
         <v>22</v>
@@ -1977,19 +1991,19 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F32" s="3">
         <v>507</v>
@@ -2010,7 +2024,7 @@
         <v>97967.88</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="M32" s="3">
         <v>22</v>
@@ -2024,19 +2038,19 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F33" s="3">
         <v>339</v>
@@ -2057,7 +2071,7 @@
         <v>65505.15</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="M33" s="3">
         <v>22</v>
@@ -2071,19 +2085,19 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F34" s="3">
         <v>93</v>
@@ -2104,7 +2118,7 @@
         <v>3652.53</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M34" s="3">
         <v>22</v>
@@ -2118,19 +2132,19 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F35" s="3">
         <v>226</v>
@@ -2151,7 +2165,7 @@
         <v>17041.99</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M35" s="3">
         <v>22</v>
@@ -2165,19 +2179,19 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F36" s="3">
         <v>675</v>
@@ -2198,7 +2212,7 @@
         <v>57262.22</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="M36" s="3">
         <v>22</v>
@@ -2212,19 +2226,19 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F37" s="3">
         <v>35</v>
@@ -2245,7 +2259,7 @@
         <v>4178.81</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="M37" s="3">
         <v>22</v>
@@ -2259,19 +2273,19 @@
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F38" s="3">
         <v>74</v>
@@ -2292,7 +2306,7 @@
         <v>17670.38</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M38" s="3">
         <v>22</v>
@@ -2306,19 +2320,19 @@
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F39" s="3">
         <v>24</v>
@@ -2339,7 +2353,7 @@
         <v>5730.94</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M39" s="3">
         <v>22</v>
@@ -2353,19 +2367,19 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F40" s="3">
         <v>45</v>
@@ -2386,7 +2400,7 @@
         <v>6715.94</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="M40" s="3">
         <v>22</v>

</xml_diff>

<commit_message>
Add warehouse column variations including typo መጋዝን
</commit_message>
<xml_diff>
--- a/Tender_3_Groups.xlsx
+++ b/Tender_3_Groups.xlsx
@@ -1,12 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="18600" windowHeight="6800"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="ጨረታ" state="visible" r:id="rId4"/>
+    <sheet name="ጨረታ" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -364,20 +380,181 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="22">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <family val="2"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -387,10 +564,197 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -399,15 +763,265 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -415,17 +1029,61 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -747,14 +1405,14 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:O40"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
@@ -766,7 +1424,7 @@
     <col min="12" max="15" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -774,7 +1432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -782,7 +1440,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -790,7 +1448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -798,7 +1456,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -806,7 +1464,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -814,7 +1472,7 @@
         <v>157.098</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -861,7 +1519,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -908,7 +1566,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15">
       <c r="A9" s="2" t="s">
         <v>32</v>
       </c>
@@ -955,7 +1613,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15">
       <c r="A10" s="2" t="s">
         <v>32</v>
       </c>
@@ -1002,7 +1660,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15">
       <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
@@ -1049,7 +1707,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15">
       <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
@@ -1096,7 +1754,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15">
       <c r="A13" s="2" t="s">
         <v>32</v>
       </c>
@@ -1143,7 +1801,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -1190,7 +1848,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -1237,7 +1895,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15">
       <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
@@ -1284,7 +1942,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15">
       <c r="A17" s="2" t="s">
         <v>32</v>
       </c>
@@ -1331,7 +1989,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15">
       <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
@@ -1378,7 +2036,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15">
       <c r="A19" s="2" t="s">
         <v>59</v>
       </c>
@@ -1425,7 +2083,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15">
       <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
@@ -1472,7 +2130,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15">
       <c r="A21" s="2" t="s">
         <v>32</v>
       </c>
@@ -1519,7 +2177,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15">
       <c r="A22" s="2" t="s">
         <v>32</v>
       </c>
@@ -1566,7 +2224,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15">
       <c r="A23" s="2" t="s">
         <v>32</v>
       </c>
@@ -1613,7 +2271,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15">
       <c r="A24" s="2" t="s">
         <v>32</v>
       </c>
@@ -1660,7 +2318,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15">
       <c r="A25" s="2" t="s">
         <v>32</v>
       </c>
@@ -1707,7 +2365,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15">
       <c r="A26" s="2" t="s">
         <v>32</v>
       </c>
@@ -1754,7 +2412,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15">
       <c r="A27" s="2" t="s">
         <v>32</v>
       </c>
@@ -1801,7 +2459,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15">
       <c r="A28" s="2" t="s">
         <v>32</v>
       </c>
@@ -1848,7 +2506,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15">
       <c r="A29" s="2" t="s">
         <v>32</v>
       </c>
@@ -1895,7 +2553,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15">
       <c r="A30" s="2" t="s">
         <v>89</v>
       </c>
@@ -1942,7 +2600,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15">
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
@@ -1989,7 +2647,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15">
       <c r="A32" s="2" t="s">
         <v>32</v>
       </c>
@@ -2036,7 +2694,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
@@ -2083,7 +2741,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -2130,7 +2788,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15">
       <c r="A35" s="2" t="s">
         <v>32</v>
       </c>
@@ -2177,7 +2835,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15">
       <c r="A36" s="2" t="s">
         <v>32</v>
       </c>
@@ -2224,7 +2882,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15">
       <c r="A37" s="2" t="s">
         <v>32</v>
       </c>
@@ -2271,7 +2929,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15">
       <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
@@ -2318,7 +2976,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15">
       <c r="A39" s="2" t="s">
         <v>32</v>
       </c>
@@ -2365,7 +3023,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15">
       <c r="A40" s="2" t="s">
         <v>32</v>
       </c>
@@ -2414,6 +3072,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Excel export: remove repeated columns, use sequential numbers in ተ.ቁ
</commit_message>
<xml_diff>
--- a/Tender_3_Groups.xlsx
+++ b/Tender_3_Groups.xlsx
@@ -83,7 +83,7 @@
     <t>መጋዘን 2</t>
   </si>
   <si>
-    <t>መጋዝን 3</t>
+    <t>መጋዘን 3</t>
   </si>
   <si>
     <t>ጠቅላላ ድምር</t>
@@ -387,7 +387,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -398,13 +398,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -878,148 +871,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>